<commit_message>
Coal to Hard coal for HOBcoal unit.
</commit_message>
<xml_diff>
--- a/src_files/data_files/unittypedata_maf2020.xlsx
+++ b/src_files/data_files/unittypedata_maf2020.xlsx
@@ -1,22 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29530"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Backbone\north_european_model\src_files\data_files\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D77E2D64-18B5-471D-8884-762A5044D504}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6E2F3DD8-0DF0-4707-873A-27C83B504C12}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="-1800" windowWidth="29040" windowHeight="17520" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="unittypedata" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">unittypedata!$C$1:$AK$91</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">unittypedata!$C$1:$AK$95</definedName>
     <definedName name="Bottom">OFFSET(#REF!,1,0,COUNT(#REF!),1)</definedName>
     <definedName name="fd">OFFSET(#REF!,1,0,COUNT(#REF!),1)</definedName>
     <definedName name="Labels">OFFSET(Bottom,0,-1)</definedName>
@@ -68,7 +68,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="566" uniqueCount="259">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="566" uniqueCount="258">
   <si>
     <t>vomCosts</t>
   </si>
@@ -824,9 +824,6 @@
   </si>
   <si>
     <t>HOBcoal</t>
-  </si>
-  <si>
-    <t>Coal</t>
   </si>
   <si>
     <t>Coal CHP extraction</t>
@@ -1253,6 +1250,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <sheetPr filterMode="1"/>
   <dimension ref="A1:AN95"/>
   <sheetFormatPr defaultColWidth="8.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -1399,7 +1397,7 @@
         <v>247</v>
       </c>
     </row>
-    <row r="2" spans="1:38" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:38" hidden="1" x14ac:dyDescent="0.25">
       <c r="A2" s="11" t="s">
         <v>220</v>
       </c>
@@ -1462,7 +1460,7 @@
       </c>
       <c r="AK2" s="2"/>
     </row>
-    <row r="3" spans="1:38" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:38" hidden="1" x14ac:dyDescent="0.25">
       <c r="A3" s="11" t="s">
         <v>220</v>
       </c>
@@ -1524,7 +1522,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:38" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:38" hidden="1" x14ac:dyDescent="0.25">
       <c r="A4" s="11" t="s">
         <v>220</v>
       </c>
@@ -1559,7 +1557,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:38" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:38" s="2" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A5" s="11" t="s">
         <v>220</v>
       </c>
@@ -1638,7 +1636,7 @@
       </c>
       <c r="AK5" s="4"/>
     </row>
-    <row r="6" spans="1:38" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:38" s="2" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A6" s="11" t="s">
         <v>220</v>
       </c>
@@ -1715,7 +1713,7 @@
       <c r="AJ6" s="5"/>
       <c r="AK6" s="4"/>
     </row>
-    <row r="7" spans="1:38" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:38" s="2" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A7" s="11" t="s">
         <v>220</v>
       </c>
@@ -1794,7 +1792,7 @@
       </c>
       <c r="AK7" s="7"/>
     </row>
-    <row r="8" spans="1:38" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:38" s="2" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A8" s="11" t="s">
         <v>220</v>
       </c>
@@ -1871,7 +1869,7 @@
       <c r="AJ8" s="7"/>
       <c r="AK8" s="7"/>
     </row>
-    <row r="9" spans="1:38" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:38" hidden="1" x14ac:dyDescent="0.25">
       <c r="A9" s="11" t="s">
         <v>220</v>
       </c>
@@ -1930,7 +1928,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:38" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:38" hidden="1" x14ac:dyDescent="0.25">
       <c r="A10" s="11" t="s">
         <v>220</v>
       </c>
@@ -2007,7 +2005,7 @@
       <c r="AJ10" s="2"/>
       <c r="AK10" s="2"/>
     </row>
-    <row r="11" spans="1:38" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:38" hidden="1" x14ac:dyDescent="0.25">
       <c r="A11" s="11" t="s">
         <v>220</v>
       </c>
@@ -2066,7 +2064,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:38" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:38" s="2" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A12" s="11" t="s">
         <v>220</v>
       </c>
@@ -2143,7 +2141,7 @@
       <c r="AJ12"/>
       <c r="AK12"/>
     </row>
-    <row r="13" spans="1:38" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:38" hidden="1" x14ac:dyDescent="0.25">
       <c r="A13" s="11" t="s">
         <v>220</v>
       </c>
@@ -2202,7 +2200,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:38" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:38" s="2" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A14" s="11" t="s">
         <v>220</v>
       </c>
@@ -2264,7 +2262,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="15" spans="1:38" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:38" s="2" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A15" s="11" t="s">
         <v>220</v>
       </c>
@@ -2326,7 +2324,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="16" spans="1:38" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:38" s="2" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A16" s="11" t="s">
         <v>220</v>
       </c>
@@ -2403,7 +2401,7 @@
       <c r="AJ16"/>
       <c r="AK16"/>
     </row>
-    <row r="17" spans="1:37" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:37" hidden="1" x14ac:dyDescent="0.25">
       <c r="A17" s="11" t="s">
         <v>220</v>
       </c>
@@ -2465,7 +2463,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="18" spans="1:37" s="8" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:37" s="8" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A18" s="11" t="s">
         <v>220</v>
       </c>
@@ -2542,7 +2540,7 @@
       <c r="AJ18" s="4"/>
       <c r="AK18" s="4"/>
     </row>
-    <row r="19" spans="1:37" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:37" hidden="1" x14ac:dyDescent="0.25">
       <c r="A19" s="11" t="s">
         <v>220</v>
       </c>
@@ -2619,7 +2617,7 @@
       <c r="AJ19" s="4"/>
       <c r="AK19" s="4"/>
     </row>
-    <row r="20" spans="1:37" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:37" hidden="1" x14ac:dyDescent="0.25">
       <c r="A20" s="11" t="s">
         <v>220</v>
       </c>
@@ -2678,7 +2676,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="21" spans="1:37" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:37" hidden="1" x14ac:dyDescent="0.25">
       <c r="A21" s="11" t="s">
         <v>220</v>
       </c>
@@ -2737,7 +2735,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="22" spans="1:37" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:37" hidden="1" x14ac:dyDescent="0.25">
       <c r="A22" s="11" t="s">
         <v>220</v>
       </c>
@@ -2814,7 +2812,7 @@
       <c r="AJ22" s="4"/>
       <c r="AK22" s="4"/>
     </row>
-    <row r="23" spans="1:37" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:37" hidden="1" x14ac:dyDescent="0.25">
       <c r="A23" s="11" t="s">
         <v>220</v>
       </c>
@@ -2903,7 +2901,7 @@
       <c r="AJ23" s="2"/>
       <c r="AK23" s="2"/>
     </row>
-    <row r="24" spans="1:37" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:37" hidden="1" x14ac:dyDescent="0.25">
       <c r="A24" s="11" t="s">
         <v>220</v>
       </c>
@@ -2980,7 +2978,7 @@
         <v>57.17</v>
       </c>
     </row>
-    <row r="25" spans="1:37" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:37" hidden="1" x14ac:dyDescent="0.25">
       <c r="A25" s="11" t="s">
         <v>220</v>
       </c>
@@ -3069,7 +3067,7 @@
       <c r="AJ25" s="2"/>
       <c r="AK25" s="2"/>
     </row>
-    <row r="26" spans="1:37" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:37" hidden="1" x14ac:dyDescent="0.25">
       <c r="A26" s="11" t="s">
         <v>220</v>
       </c>
@@ -3152,7 +3150,7 @@
         <v>57.17</v>
       </c>
     </row>
-    <row r="27" spans="1:37" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:37" hidden="1" x14ac:dyDescent="0.25">
       <c r="A27" s="11" t="s">
         <v>220</v>
       </c>
@@ -3245,7 +3243,7 @@
       <c r="AJ27" s="10"/>
       <c r="AK27" s="10"/>
     </row>
-    <row r="28" spans="1:37" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:37" hidden="1" x14ac:dyDescent="0.25">
       <c r="A28" s="11" t="s">
         <v>220</v>
       </c>
@@ -3320,7 +3318,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="29" spans="1:37" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:37" hidden="1" x14ac:dyDescent="0.25">
       <c r="A29" s="11" t="s">
         <v>220</v>
       </c>
@@ -3399,7 +3397,7 @@
       </c>
       <c r="AK29" s="4"/>
     </row>
-    <row r="30" spans="1:37" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:37" hidden="1" x14ac:dyDescent="0.25">
       <c r="A30" s="11" t="s">
         <v>220</v>
       </c>
@@ -3476,7 +3474,7 @@
       <c r="AJ30" s="5"/>
       <c r="AK30" s="4"/>
     </row>
-    <row r="31" spans="1:37" s="10" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:37" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A31" s="11" t="s">
         <v>220</v>
       </c>
@@ -3563,7 +3561,7 @@
       <c r="AJ31" s="2"/>
       <c r="AK31" s="2"/>
     </row>
-    <row r="32" spans="1:37" s="10" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:37" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A32" s="11" t="s">
         <v>220</v>
       </c>
@@ -3652,7 +3650,7 @@
       <c r="AJ32"/>
       <c r="AK32"/>
     </row>
-    <row r="33" spans="1:37" s="8" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:37" s="8" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A33" s="11" t="s">
         <v>220</v>
       </c>
@@ -3739,7 +3737,7 @@
       <c r="AJ33" s="2"/>
       <c r="AK33" s="2"/>
     </row>
-    <row r="34" spans="1:37" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:37" hidden="1" x14ac:dyDescent="0.25">
       <c r="A34" s="11" t="s">
         <v>220</v>
       </c>
@@ -3816,7 +3814,7 @@
         <v>93.97</v>
       </c>
     </row>
-    <row r="35" spans="1:37" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:37" hidden="1" x14ac:dyDescent="0.25">
       <c r="A35" s="11" t="s">
         <v>220</v>
       </c>
@@ -3905,7 +3903,7 @@
       <c r="AJ35" s="2"/>
       <c r="AK35" s="2"/>
     </row>
-    <row r="36" spans="1:37" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:37" s="2" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A36" s="11" t="s">
         <v>220</v>
       </c>
@@ -3979,7 +3977,7 @@
         <v>81.44</v>
       </c>
     </row>
-    <row r="37" spans="1:37" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:37" s="2" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A37" s="11" t="s">
         <v>220</v>
       </c>
@@ -4068,7 +4066,7 @@
       <c r="AJ37"/>
       <c r="AK37"/>
     </row>
-    <row r="38" spans="1:37" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:37" s="2" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A38" s="11" t="s">
         <v>220</v>
       </c>
@@ -4147,7 +4145,7 @@
       </c>
       <c r="AK38" s="7"/>
     </row>
-    <row r="39" spans="1:37" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:37" hidden="1" x14ac:dyDescent="0.25">
       <c r="A39" s="11" t="s">
         <v>220</v>
       </c>
@@ -4224,7 +4222,7 @@
       <c r="AJ39" s="7"/>
       <c r="AK39" s="7"/>
     </row>
-    <row r="40" spans="1:37" s="8" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:37" s="8" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A40" s="11" t="s">
         <v>220</v>
       </c>
@@ -4317,7 +4315,7 @@
       <c r="AJ40"/>
       <c r="AK40"/>
     </row>
-    <row r="41" spans="1:37" s="9" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:37" s="9" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A41" s="11" t="s">
         <v>220</v>
       </c>
@@ -4412,7 +4410,7 @@
       <c r="AJ41"/>
       <c r="AK41" s="2"/>
     </row>
-    <row r="42" spans="1:37" s="8" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:37" s="8" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A42" s="11" t="s">
         <v>220</v>
       </c>
@@ -4507,7 +4505,7 @@
       <c r="AJ42"/>
       <c r="AK42" s="2"/>
     </row>
-    <row r="43" spans="1:37" s="7" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:37" s="7" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A43" s="11" t="s">
         <v>220</v>
       </c>
@@ -4588,7 +4586,7 @@
       </c>
       <c r="AK43" s="2"/>
     </row>
-    <row r="44" spans="1:37" s="8" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:37" s="8" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A44" s="11" t="s">
         <v>220</v>
       </c>
@@ -4665,7 +4663,7 @@
       <c r="AJ44" s="2"/>
       <c r="AK44" s="2"/>
     </row>
-    <row r="45" spans="1:37" s="8" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:37" s="8" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A45" s="11" t="s">
         <v>220</v>
       </c>
@@ -4742,7 +4740,7 @@
       <c r="AJ45" s="2"/>
       <c r="AK45" s="2"/>
     </row>
-    <row r="46" spans="1:37" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:37" hidden="1" x14ac:dyDescent="0.25">
       <c r="A46" s="11" t="s">
         <v>220</v>
       </c>
@@ -4829,7 +4827,7 @@
       <c r="AJ46" s="7"/>
       <c r="AK46" s="7"/>
     </row>
-    <row r="47" spans="1:37" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:37" hidden="1" x14ac:dyDescent="0.25">
       <c r="A47" s="11" t="s">
         <v>220</v>
       </c>
@@ -4916,7 +4914,7 @@
       <c r="AJ47" s="8"/>
       <c r="AK47" s="8"/>
     </row>
-    <row r="48" spans="1:37" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:37" hidden="1" x14ac:dyDescent="0.25">
       <c r="A48" s="11" t="s">
         <v>220</v>
       </c>
@@ -5003,7 +5001,7 @@
       <c r="AJ48" s="8"/>
       <c r="AK48" s="8"/>
     </row>
-    <row r="49" spans="1:37" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:37" hidden="1" x14ac:dyDescent="0.25">
       <c r="A49" s="11" t="s">
         <v>220</v>
       </c>
@@ -5088,7 +5086,7 @@
       <c r="AJ49" s="8"/>
       <c r="AK49" s="8"/>
     </row>
-    <row r="50" spans="1:37" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:37" hidden="1" x14ac:dyDescent="0.25">
       <c r="A50" s="11" t="s">
         <v>220</v>
       </c>
@@ -5177,7 +5175,7 @@
       <c r="AJ50" s="2"/>
       <c r="AK50" s="2"/>
     </row>
-    <row r="51" spans="1:37" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:37" hidden="1" x14ac:dyDescent="0.25">
       <c r="A51" s="11" t="s">
         <v>220</v>
       </c>
@@ -5254,7 +5252,7 @@
         <v>93.97</v>
       </c>
     </row>
-    <row r="52" spans="1:37" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:37" hidden="1" x14ac:dyDescent="0.25">
       <c r="A52" s="11" t="s">
         <v>220</v>
       </c>
@@ -5341,7 +5339,7 @@
       <c r="AJ52" s="2"/>
       <c r="AK52" s="2"/>
     </row>
-    <row r="53" spans="1:37" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:37" s="2" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A53" s="11" t="s">
         <v>220</v>
       </c>
@@ -5420,7 +5418,7 @@
       </c>
       <c r="AK53" s="7"/>
     </row>
-    <row r="54" spans="1:37" s="4" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:37" s="4" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A54" s="11" t="s">
         <v>220</v>
       </c>
@@ -5497,7 +5495,7 @@
       <c r="AJ54" s="7"/>
       <c r="AK54" s="7"/>
     </row>
-    <row r="55" spans="1:37" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:37" s="2" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A55" s="11" t="s">
         <v>220</v>
       </c>
@@ -5575,7 +5573,7 @@
         <v>93.97</v>
       </c>
     </row>
-    <row r="56" spans="1:37" s="4" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:37" s="4" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A56" s="11" t="s">
         <v>220</v>
       </c>
@@ -5664,7 +5662,7 @@
       <c r="AJ56" s="2"/>
       <c r="AK56" s="2"/>
     </row>
-    <row r="57" spans="1:37" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:37" hidden="1" x14ac:dyDescent="0.25">
       <c r="A57" s="11" t="s">
         <v>220</v>
       </c>
@@ -5741,7 +5739,7 @@
         <v>81.44</v>
       </c>
     </row>
-    <row r="58" spans="1:37" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:37" hidden="1" x14ac:dyDescent="0.25">
       <c r="A58" s="11" t="s">
         <v>220</v>
       </c>
@@ -5819,7 +5817,7 @@
         <v>93.97</v>
       </c>
     </row>
-    <row r="59" spans="1:37" s="4" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:37" s="4" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A59" s="11" t="s">
         <v>220</v>
       </c>
@@ -5908,7 +5906,7 @@
       <c r="AJ59"/>
       <c r="AK59"/>
     </row>
-    <row r="60" spans="1:37" s="4" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:37" s="4" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A60" s="11" t="s">
         <v>220</v>
       </c>
@@ -5997,7 +5995,7 @@
       <c r="AJ60"/>
       <c r="AK60"/>
     </row>
-    <row r="61" spans="1:37" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:37" s="2" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A61" s="11" t="s">
         <v>220</v>
       </c>
@@ -6080,7 +6078,7 @@
         <v>81.44</v>
       </c>
     </row>
-    <row r="62" spans="1:37" s="4" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:37" s="4" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A62" s="11" t="s">
         <v>220</v>
       </c>
@@ -6157,7 +6155,7 @@
       <c r="AJ62"/>
       <c r="AK62"/>
     </row>
-    <row r="63" spans="1:37" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:37" s="2" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A63" s="11" t="s">
         <v>220</v>
       </c>
@@ -6244,7 +6242,7 @@
       <c r="AJ63"/>
       <c r="AK63"/>
     </row>
-    <row r="64" spans="1:37" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:37" s="2" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A64" s="11" t="s">
         <v>220</v>
       </c>
@@ -6333,7 +6331,7 @@
       <c r="AJ64"/>
       <c r="AK64"/>
     </row>
-    <row r="65" spans="1:40" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:40" s="2" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A65" s="11" t="s">
         <v>220</v>
       </c>
@@ -6422,7 +6420,7 @@
       <c r="AJ65"/>
       <c r="AK65"/>
     </row>
-    <row r="66" spans="1:40" s="4" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:40" s="4" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A66" s="11" t="s">
         <v>220</v>
       </c>
@@ -6511,7 +6509,7 @@
       <c r="AJ66"/>
       <c r="AK66"/>
     </row>
-    <row r="67" spans="1:40" s="4" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:40" s="4" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A67" s="11" t="s">
         <v>220</v>
       </c>
@@ -6600,7 +6598,7 @@
       <c r="AJ67"/>
       <c r="AK67"/>
     </row>
-    <row r="68" spans="1:40" s="4" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:40" s="4" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A68" s="11" t="s">
         <v>220</v>
       </c>
@@ -6689,7 +6687,7 @@
       <c r="AJ68"/>
       <c r="AK68"/>
     </row>
-    <row r="69" spans="1:40" s="4" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:40" s="4" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A69" s="11" t="s">
         <v>220</v>
       </c>
@@ -6778,7 +6776,7 @@
       <c r="AJ69"/>
       <c r="AK69"/>
     </row>
-    <row r="70" spans="1:40" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:40" hidden="1" x14ac:dyDescent="0.25">
       <c r="A70" s="11" t="s">
         <v>220</v>
       </c>
@@ -6855,7 +6853,7 @@
       <c r="AM70" s="4"/>
       <c r="AN70" s="4"/>
     </row>
-    <row r="71" spans="1:40" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:40" hidden="1" x14ac:dyDescent="0.25">
       <c r="A71" s="11" t="s">
         <v>220</v>
       </c>
@@ -6932,7 +6930,7 @@
         <v>61.86</v>
       </c>
     </row>
-    <row r="72" spans="1:40" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:40" s="2" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A72" s="11" t="s">
         <v>220</v>
       </c>
@@ -7021,7 +7019,7 @@
       <c r="AJ72"/>
       <c r="AK72"/>
     </row>
-    <row r="73" spans="1:40" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:40" s="2" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A73" s="11" t="s">
         <v>220</v>
       </c>
@@ -7110,7 +7108,7 @@
       <c r="AJ73"/>
       <c r="AK73"/>
     </row>
-    <row r="74" spans="1:40" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:40" s="2" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A74" s="11" t="s">
         <v>220</v>
       </c>
@@ -7202,7 +7200,7 @@
       <c r="AJ74"/>
       <c r="AK74"/>
     </row>
-    <row r="75" spans="1:40" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:40" hidden="1" x14ac:dyDescent="0.25">
       <c r="A75" s="11" t="s">
         <v>220</v>
       </c>
@@ -7279,7 +7277,7 @@
       <c r="AJ75" s="2"/>
       <c r="AK75" s="2"/>
     </row>
-    <row r="76" spans="1:40" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:40" hidden="1" x14ac:dyDescent="0.25">
       <c r="A76" s="11" t="s">
         <v>220</v>
       </c>
@@ -7358,7 +7356,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="77" spans="1:40" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:40" hidden="1" x14ac:dyDescent="0.25">
       <c r="A77" s="11" t="s">
         <v>220</v>
       </c>
@@ -7435,7 +7433,7 @@
       <c r="AJ77" s="2"/>
       <c r="AK77" s="2"/>
     </row>
-    <row r="78" spans="1:40" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:40" s="2" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A78" s="11" t="s">
         <v>220</v>
       </c>
@@ -7512,7 +7510,7 @@
       <c r="AJ78"/>
       <c r="AK78"/>
     </row>
-    <row r="79" spans="1:40" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:40" s="2" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A79" s="11" t="s">
         <v>220</v>
       </c>
@@ -7591,7 +7589,7 @@
       <c r="AJ79"/>
       <c r="AK79"/>
     </row>
-    <row r="80" spans="1:40" s="7" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:40" s="7" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A80" s="11" t="s">
         <v>220</v>
       </c>
@@ -7670,7 +7668,7 @@
       <c r="AJ80"/>
       <c r="AK80"/>
     </row>
-    <row r="81" spans="1:38" s="7" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:38" s="7" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A81" s="11" t="s">
         <v>220</v>
       </c>
@@ -7749,7 +7747,7 @@
       <c r="AJ81" s="2"/>
       <c r="AK81" s="2"/>
     </row>
-    <row r="82" spans="1:38" s="7" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:38" s="7" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A82" s="11" t="s">
         <v>220</v>
       </c>
@@ -7828,7 +7826,7 @@
       <c r="AJ82"/>
       <c r="AK82"/>
     </row>
-    <row r="83" spans="1:38" s="7" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:38" s="7" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A83" s="11" t="s">
         <v>220</v>
       </c>
@@ -7907,7 +7905,7 @@
       <c r="AJ83"/>
       <c r="AK83"/>
     </row>
-    <row r="84" spans="1:38" s="7" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:38" s="7" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A84" s="11" t="s">
         <v>220</v>
       </c>
@@ -8000,7 +7998,7 @@
       <c r="AJ84" s="8"/>
       <c r="AK84" s="8"/>
     </row>
-    <row r="85" spans="1:38" s="7" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:38" s="7" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A85" s="11" t="s">
         <v>220</v>
       </c>
@@ -8093,7 +8091,7 @@
       <c r="AJ85" s="8"/>
       <c r="AK85" s="8"/>
     </row>
-    <row r="86" spans="1:38" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:38" hidden="1" x14ac:dyDescent="0.25">
       <c r="A86" s="11" t="s">
         <v>220</v>
       </c>
@@ -8184,7 +8182,7 @@
       <c r="AJ86" s="8"/>
       <c r="AK86" s="8"/>
     </row>
-    <row r="87" spans="1:38" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:38" hidden="1" x14ac:dyDescent="0.25">
       <c r="A87" s="11" t="s">
         <v>220</v>
       </c>
@@ -8277,7 +8275,7 @@
       <c r="AJ87" s="10"/>
       <c r="AK87" s="10"/>
     </row>
-    <row r="88" spans="1:38" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:38" hidden="1" x14ac:dyDescent="0.25">
       <c r="A88" s="11" t="s">
         <v>220</v>
       </c>
@@ -8356,7 +8354,7 @@
       </c>
       <c r="AK88" s="4"/>
     </row>
-    <row r="89" spans="1:38" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:38" hidden="1" x14ac:dyDescent="0.25">
       <c r="A89" s="11" t="s">
         <v>220</v>
       </c>
@@ -8435,7 +8433,7 @@
       </c>
       <c r="AK89" s="2"/>
     </row>
-    <row r="90" spans="1:38" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:38" hidden="1" x14ac:dyDescent="0.25">
       <c r="A90" s="11" t="s">
         <v>220</v>
       </c>
@@ -8512,7 +8510,7 @@
       <c r="AJ90" s="4"/>
       <c r="AK90" s="4"/>
     </row>
-    <row r="91" spans="1:38" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:38" hidden="1" x14ac:dyDescent="0.25">
       <c r="A91" t="s">
         <v>220</v>
       </c>
@@ -8609,7 +8607,7 @@
         <v>249</v>
       </c>
       <c r="J92" t="s">
-        <v>252</v>
+        <v>17</v>
       </c>
       <c r="K92" t="s">
         <v>221</v>
@@ -8666,7 +8664,7 @@
         <v>0.05</v>
       </c>
     </row>
-    <row r="93" spans="1:38" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:38" hidden="1" x14ac:dyDescent="0.25">
       <c r="A93" t="s">
         <v>220</v>
       </c>
@@ -8674,10 +8672,10 @@
         <v>1</v>
       </c>
       <c r="C93" t="s">
+        <v>252</v>
+      </c>
+      <c r="D93" t="s">
         <v>253</v>
-      </c>
-      <c r="D93" t="s">
-        <v>254</v>
       </c>
       <c r="I93" t="s">
         <v>249</v>
@@ -8752,7 +8750,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="94" spans="1:38" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:38" hidden="1" x14ac:dyDescent="0.25">
       <c r="A94" t="s">
         <v>220</v>
       </c>
@@ -8760,10 +8758,10 @@
         <v>1</v>
       </c>
       <c r="C94" t="s">
+        <v>254</v>
+      </c>
+      <c r="D94" t="s">
         <v>255</v>
-      </c>
-      <c r="D94" t="s">
-        <v>256</v>
       </c>
       <c r="J94" t="s">
         <v>54</v>
@@ -8835,7 +8833,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="95" spans="1:38" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:38" hidden="1" x14ac:dyDescent="0.25">
       <c r="A95" t="s">
         <v>220</v>
       </c>
@@ -8843,10 +8841,10 @@
         <v>1</v>
       </c>
       <c r="C95" t="s">
+        <v>256</v>
+      </c>
+      <c r="D95" t="s">
         <v>257</v>
-      </c>
-      <c r="D95" t="s">
-        <v>258</v>
       </c>
       <c r="I95" t="s">
         <v>249</v>
@@ -8922,7 +8920,12 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="C1:AK91" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <autoFilter ref="C1:AK95" xr:uid="{00000000-0001-0000-0000-000000000000}">
+    <filterColumn colId="1">
+      <filters>
+        <filter val="HOBcoal"/>
+      </filters>
+    </filterColumn>
     <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="C2:AK91">
       <sortCondition descending="1" ref="D1:D91"/>
     </sortState>

</xml_diff>